<commit_message>
Test 1 à 7
</commit_message>
<xml_diff>
--- a/Exigences_US_CT.xlsx
+++ b/Exigences_US_CT.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fanle\Documents\Formation SOGETI\z-EDC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fanle\Documents\Formation SOGETI\z-EDC\projet\projet_tutore_LECLERC_FANNY\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CEBFE73-2AE0-45A1-B22E-F8E3DBB8D917}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
@@ -1132,7 +1132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1209,59 +1209,8 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1284,86 +1233,100 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="8">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="darkUp">
-          <fgColor theme="0" tint="-0.34998626667073579"/>
-          <bgColor theme="2"/>
-        </patternFill>
-      </fill>
-    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1389,6 +1352,40 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+      </font>
+      <fill>
+        <patternFill patternType="darkUp">
+          <fgColor theme="0" tint="-0.34998626667073579"/>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1706,91 +1703,91 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="27" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="44"/>
+      <c r="A2" s="27"/>
     </row>
     <row r="3" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="44" t="s">
+      <c r="A3" s="27" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="44" t="s">
+      <c r="A4" s="27" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="44" t="s">
+      <c r="A5" s="27" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="44" t="s">
+      <c r="A6" s="27" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="44" t="s">
+      <c r="A7" s="27" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="44" t="s">
+      <c r="A8" s="27" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="44" t="s">
+      <c r="A9" s="27" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="44"/>
+      <c r="A10" s="27"/>
     </row>
     <row r="11" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="44" t="s">
+      <c r="A11" s="27" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="44" t="s">
+      <c r="A12" s="27" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="44" t="s">
+      <c r="A13" s="27" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="14" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="44" t="s">
+      <c r="A14" s="27" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="15" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="44"/>
+      <c r="A15" s="27"/>
     </row>
     <row r="16" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="44" t="s">
+      <c r="A16" s="27" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="44" t="s">
+      <c r="A17" s="27" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="44" t="s">
+      <c r="A18" s="27" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="19" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="44"/>
+      <c r="A19" s="27"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1806,119 +1803,119 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="27" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="27" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="44" t="s">
+      <c r="A3" s="27" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="44" t="s">
+      <c r="A4" s="27" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="44" t="s">
+      <c r="A5" s="27" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="44" t="s">
+      <c r="A6" s="27" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="44" t="s">
+      <c r="A7" s="27" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="44" t="s">
+      <c r="A9" s="27" t="s">
         <v>98</v>
       </c>
-      <c r="O9" s="49"/>
+      <c r="O9" s="32"/>
     </row>
     <row r="10" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A10" s="46" t="s">
+      <c r="A10" s="29" t="s">
         <v>46</v>
       </c>
-      <c r="B10" s="47"/>
-      <c r="C10" s="46" t="s">
+      <c r="B10" s="30"/>
+      <c r="C10" s="29" t="s">
         <v>47</v>
       </c>
-      <c r="D10" s="47"/>
-      <c r="E10" s="46" t="s">
+      <c r="D10" s="30"/>
+      <c r="E10" s="29" t="s">
         <v>48</v>
       </c>
-      <c r="F10" s="47"/>
-      <c r="G10" s="46" t="s">
+      <c r="F10" s="30"/>
+      <c r="G10" s="29" t="s">
         <v>73</v>
       </c>
-      <c r="H10" s="47"/>
-      <c r="I10" s="46" t="s">
+      <c r="H10" s="30"/>
+      <c r="I10" s="29" t="s">
         <v>49</v>
       </c>
-      <c r="J10" s="47" t="s">
+      <c r="J10" s="30" t="s">
         <v>97</v>
       </c>
-      <c r="K10" s="46" t="s">
+      <c r="K10" s="29" t="s">
         <v>50</v>
       </c>
-      <c r="L10" s="47"/>
-      <c r="M10" s="46" t="s">
+      <c r="L10" s="30"/>
+      <c r="M10" s="29" t="s">
         <v>51</v>
       </c>
-      <c r="N10" s="49" t="s">
+      <c r="N10" s="32" t="s">
         <v>87</v>
       </c>
-      <c r="O10" s="49" t="s">
+      <c r="O10" s="32" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="11" spans="1:15" ht="230.4" x14ac:dyDescent="0.3">
-      <c r="A11" s="49" t="s">
+      <c r="A11" s="32" t="s">
         <v>74</v>
       </c>
-      <c r="B11" s="47"/>
-      <c r="C11" s="47" t="s">
+      <c r="B11" s="30"/>
+      <c r="C11" s="30" t="s">
         <v>96</v>
       </c>
-      <c r="D11" s="47"/>
-      <c r="E11" s="47" t="s">
+      <c r="D11" s="30"/>
+      <c r="E11" s="30" t="s">
         <v>66</v>
       </c>
-      <c r="F11" s="47"/>
-      <c r="G11" s="47"/>
-      <c r="H11" s="47"/>
-      <c r="I11" s="47"/>
-      <c r="J11" s="49" t="s">
+      <c r="F11" s="30"/>
+      <c r="G11" s="30"/>
+      <c r="H11" s="30"/>
+      <c r="I11" s="30"/>
+      <c r="J11" s="32" t="s">
         <v>77</v>
       </c>
-      <c r="K11" s="47" t="s">
+      <c r="K11" s="30" t="s">
         <v>69</v>
       </c>
-      <c r="L11" s="47"/>
-      <c r="M11" s="47" t="s">
+      <c r="L11" s="30"/>
+      <c r="M11" s="30" t="s">
         <v>70</v>
       </c>
-      <c r="N11" s="50" t="s">
+      <c r="N11" s="33" t="s">
         <v>88</v>
       </c>
-      <c r="O11" s="48"/>
+      <c r="O11" s="31"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A12" s="50" t="s">
+      <c r="A12" s="33" t="s">
         <v>75</v>
       </c>
-      <c r="C12" s="47" t="s">
+      <c r="C12" s="30" t="s">
         <v>59</v>
       </c>
       <c r="E12" t="s">
@@ -1927,7 +1924,7 @@
       <c r="G12" t="s">
         <v>58</v>
       </c>
-      <c r="J12" s="50" t="s">
+      <c r="J12" s="33" t="s">
         <v>78</v>
       </c>
       <c r="K12" t="s">
@@ -1936,65 +1933,65 @@
       <c r="M12" t="s">
         <v>72</v>
       </c>
-      <c r="N12" s="50" t="s">
+      <c r="N12" s="33" t="s">
         <v>89</v>
       </c>
-      <c r="O12" s="48" t="s">
+      <c r="O12" s="31" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="13" spans="1:15" ht="72" x14ac:dyDescent="0.3">
-      <c r="A13" s="50" t="s">
+      <c r="A13" s="33" t="s">
         <v>76</v>
       </c>
-      <c r="C13" s="47" t="s">
+      <c r="C13" s="30" t="s">
         <v>65</v>
       </c>
-      <c r="E13" s="48"/>
-      <c r="G13" s="49" t="s">
+      <c r="E13" s="31"/>
+      <c r="G13" s="32" t="s">
         <v>80</v>
       </c>
-      <c r="J13" s="50" t="s">
+      <c r="J13" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="K13" s="49" t="s">
+      <c r="K13" s="32" t="s">
         <v>84</v>
       </c>
-      <c r="M13" s="49" t="s">
+      <c r="M13" s="32" t="s">
         <v>90</v>
       </c>
-      <c r="O13" s="48" t="s">
+      <c r="O13" s="31" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="E14" s="48" t="s">
+      <c r="E14" s="31" t="s">
         <v>53</v>
       </c>
-      <c r="G14" s="50" t="s">
+      <c r="G14" s="33" t="s">
         <v>81</v>
       </c>
-      <c r="K14" s="50" t="s">
+      <c r="K14" s="33" t="s">
         <v>85</v>
       </c>
-      <c r="M14" s="50" t="s">
+      <c r="M14" s="33" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="C15" s="47" t="s">
+      <c r="C15" s="30" t="s">
         <v>60</v>
       </c>
-      <c r="E15" s="48" t="s">
+      <c r="E15" s="31" t="s">
         <v>63</v>
       </c>
-      <c r="G15" s="50" t="s">
+      <c r="G15" s="33" t="s">
         <v>82</v>
       </c>
-      <c r="K15" s="50" t="s">
+      <c r="K15" s="33" t="s">
         <v>86</v>
       </c>
-      <c r="M15" s="50" t="s">
+      <c r="M15" s="33" t="s">
         <v>92</v>
       </c>
     </row>
@@ -2002,10 +1999,10 @@
       <c r="C16" t="s">
         <v>61</v>
       </c>
-      <c r="E16" s="48" t="s">
+      <c r="E16" s="31" t="s">
         <v>64</v>
       </c>
-      <c r="G16" s="50" t="s">
+      <c r="G16" s="33" t="s">
         <v>83</v>
       </c>
     </row>
@@ -2018,22 +2015,22 @@
       <c r="E18" t="s">
         <v>54</v>
       </c>
-      <c r="G18" s="50" t="s">
+      <c r="G18" s="33" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="19" spans="3:7" x14ac:dyDescent="0.3">
-      <c r="C19" s="49"/>
-      <c r="E19" s="48"/>
+      <c r="C19" s="32"/>
+      <c r="E19" s="31"/>
     </row>
     <row r="20" spans="3:7" x14ac:dyDescent="0.3">
-      <c r="C20" s="50"/>
-      <c r="E20" s="48" t="s">
+      <c r="C20" s="33"/>
+      <c r="E20" s="31" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="21" spans="3:7" x14ac:dyDescent="0.3">
-      <c r="C21" s="50"/>
+      <c r="C21" s="33"/>
     </row>
     <row r="22" spans="3:7" x14ac:dyDescent="0.3">
       <c r="E22" t="s">
@@ -2041,10 +2038,10 @@
       </c>
     </row>
     <row r="23" spans="3:7" x14ac:dyDescent="0.3">
-      <c r="E23" s="48"/>
+      <c r="E23" s="31"/>
     </row>
     <row r="24" spans="3:7" x14ac:dyDescent="0.3">
-      <c r="E24" s="48" t="s">
+      <c r="E24" s="31" t="s">
         <v>57</v>
       </c>
     </row>
@@ -2119,29 +2116,29 @@
       </c>
     </row>
     <row r="2" spans="2:12" ht="51" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="59" t="s">
         <v>132</v>
       </c>
-      <c r="C2" s="32" t="s">
+      <c r="C2" s="60" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="34" t="s">
+      <c r="D2" s="52" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="34" t="s">
+      <c r="E2" s="52" t="s">
         <v>19</v>
       </c>
-      <c r="F2" s="34">
+      <c r="F2" s="52">
         <v>3</v>
       </c>
-      <c r="G2" s="34">
+      <c r="G2" s="52">
         <v>3</v>
       </c>
-      <c r="H2" s="34">
+      <c r="H2" s="52">
         <f>F2*G2</f>
         <v>9</v>
       </c>
-      <c r="I2" s="34" t="s">
+      <c r="I2" s="52" t="s">
         <v>28</v>
       </c>
       <c r="J2" s="6" t="s">
@@ -2155,14 +2152,14 @@
       </c>
     </row>
     <row r="3" spans="2:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="33"/>
-      <c r="C3" s="32"/>
-      <c r="D3" s="35"/>
-      <c r="E3" s="36"/>
-      <c r="F3" s="36"/>
-      <c r="G3" s="36"/>
-      <c r="H3" s="36"/>
-      <c r="I3" s="36"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="60"/>
+      <c r="D3" s="55"/>
+      <c r="E3" s="53"/>
+      <c r="F3" s="53"/>
+      <c r="G3" s="53"/>
+      <c r="H3" s="53"/>
+      <c r="I3" s="53"/>
       <c r="J3" s="6" t="s">
         <v>179</v>
       </c>
@@ -2174,9 +2171,9 @@
       </c>
     </row>
     <row r="4" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="33"/>
-      <c r="C4" s="32"/>
-      <c r="D4" s="35"/>
+      <c r="B4" s="59"/>
+      <c r="C4" s="60"/>
+      <c r="D4" s="55"/>
       <c r="E4" s="7" t="s">
         <v>20</v>
       </c>
@@ -2204,23 +2201,23 @@
       </c>
     </row>
     <row r="5" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="33"/>
-      <c r="C5" s="32"/>
-      <c r="D5" s="35"/>
-      <c r="E5" s="34" t="s">
+      <c r="B5" s="59"/>
+      <c r="C5" s="60"/>
+      <c r="D5" s="55"/>
+      <c r="E5" s="52" t="s">
         <v>176</v>
       </c>
-      <c r="F5" s="34">
+      <c r="F5" s="52">
         <v>2</v>
       </c>
-      <c r="G5" s="34">
+      <c r="G5" s="52">
         <v>2</v>
       </c>
-      <c r="H5" s="34">
+      <c r="H5" s="52">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="I5" s="34" t="s">
+      <c r="I5" s="52" t="s">
         <v>28</v>
       </c>
       <c r="J5" s="6" t="s">
@@ -2232,14 +2229,14 @@
       <c r="L5" s="7"/>
     </row>
     <row r="6" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="33"/>
-      <c r="C6" s="32"/>
-      <c r="D6" s="36"/>
-      <c r="E6" s="36"/>
-      <c r="F6" s="36"/>
-      <c r="G6" s="36"/>
-      <c r="H6" s="36"/>
-      <c r="I6" s="36"/>
+      <c r="B6" s="59"/>
+      <c r="C6" s="60"/>
+      <c r="D6" s="53"/>
+      <c r="E6" s="53"/>
+      <c r="F6" s="53"/>
+      <c r="G6" s="53"/>
+      <c r="H6" s="53"/>
+      <c r="I6" s="53"/>
       <c r="J6" s="6" t="s">
         <v>178</v>
       </c>
@@ -2249,9 +2246,9 @@
       <c r="L6" s="7"/>
     </row>
     <row r="7" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="33"/>
-      <c r="C7" s="32"/>
-      <c r="D7" s="34" t="s">
+      <c r="B7" s="59"/>
+      <c r="C7" s="60"/>
+      <c r="D7" s="52" t="s">
         <v>23</v>
       </c>
       <c r="E7" s="7" t="s">
@@ -2281,9 +2278,9 @@
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B8" s="33"/>
-      <c r="C8" s="32"/>
-      <c r="D8" s="35"/>
+      <c r="B8" s="59"/>
+      <c r="C8" s="60"/>
+      <c r="D8" s="55"/>
       <c r="E8" s="7" t="s">
         <v>21</v>
       </c>
@@ -2305,9 +2302,9 @@
       <c r="L8" s="12"/>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B9" s="33"/>
-      <c r="C9" s="32"/>
-      <c r="D9" s="36"/>
+      <c r="B9" s="59"/>
+      <c r="C9" s="60"/>
+      <c r="D9" s="53"/>
       <c r="E9" s="7" t="s">
         <v>122</v>
       </c>
@@ -2329,503 +2326,503 @@
       <c r="L9" s="13"/>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B10" s="33"/>
-      <c r="C10" s="55" t="s">
+      <c r="B10" s="59"/>
+      <c r="C10" s="50" t="s">
         <v>182</v>
       </c>
-      <c r="D10" s="55" t="s">
+      <c r="D10" s="50" t="s">
         <v>183</v>
       </c>
-      <c r="E10" s="56" t="s">
+      <c r="E10" s="37" t="s">
         <v>186</v>
       </c>
-      <c r="F10" s="58">
+      <c r="F10" s="36">
         <v>2</v>
       </c>
-      <c r="G10" s="58">
+      <c r="G10" s="36">
         <v>3</v>
       </c>
-      <c r="H10" s="58">
+      <c r="H10" s="36">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="I10" s="58" t="s">
+      <c r="I10" s="36" t="s">
         <v>28</v>
       </c>
-      <c r="J10" s="59" t="s">
+      <c r="J10" s="39" t="s">
         <v>191</v>
       </c>
-      <c r="K10" s="56" t="s">
+      <c r="K10" s="37" t="s">
         <v>25</v>
       </c>
-      <c r="L10" s="64"/>
+      <c r="L10" s="41"/>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B11" s="33"/>
-      <c r="C11" s="61"/>
-      <c r="D11" s="61"/>
-      <c r="E11" s="56" t="s">
+      <c r="B11" s="59"/>
+      <c r="C11" s="54"/>
+      <c r="D11" s="54"/>
+      <c r="E11" s="37" t="s">
         <v>187</v>
       </c>
-      <c r="F11" s="58">
+      <c r="F11" s="36">
         <v>2</v>
       </c>
-      <c r="G11" s="58">
+      <c r="G11" s="36">
         <v>1</v>
       </c>
-      <c r="H11" s="58">
+      <c r="H11" s="36">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="I11" s="58" t="s">
-        <v>27</v>
-      </c>
-      <c r="J11" s="59"/>
-      <c r="K11" s="56"/>
-      <c r="L11" s="64"/>
+      <c r="I11" s="36" t="s">
+        <v>27</v>
+      </c>
+      <c r="J11" s="39"/>
+      <c r="K11" s="37"/>
+      <c r="L11" s="41"/>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B12" s="33"/>
-      <c r="C12" s="61"/>
-      <c r="D12" s="61"/>
-      <c r="E12" s="55" t="s">
+      <c r="B12" s="59"/>
+      <c r="C12" s="54"/>
+      <c r="D12" s="54"/>
+      <c r="E12" s="50" t="s">
         <v>188</v>
       </c>
-      <c r="F12" s="55">
+      <c r="F12" s="50">
         <v>3</v>
       </c>
-      <c r="G12" s="55">
+      <c r="G12" s="50">
         <v>3</v>
       </c>
-      <c r="H12" s="55">
+      <c r="H12" s="50">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="I12" s="55" t="s">
+      <c r="I12" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="J12" s="59" t="s">
+      <c r="J12" s="39" t="s">
         <v>192</v>
       </c>
-      <c r="K12" s="56" t="s">
+      <c r="K12" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="L12" s="64" t="s">
+      <c r="L12" s="41" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B13" s="33"/>
-      <c r="C13" s="61"/>
-      <c r="D13" s="61"/>
-      <c r="E13" s="62"/>
-      <c r="F13" s="62"/>
-      <c r="G13" s="62"/>
-      <c r="H13" s="62"/>
-      <c r="I13" s="62"/>
-      <c r="J13" s="59" t="s">
+      <c r="B13" s="59"/>
+      <c r="C13" s="54"/>
+      <c r="D13" s="54"/>
+      <c r="E13" s="51"/>
+      <c r="F13" s="51"/>
+      <c r="G13" s="51"/>
+      <c r="H13" s="51"/>
+      <c r="I13" s="51"/>
+      <c r="J13" s="39" t="s">
         <v>193</v>
       </c>
-      <c r="K13" s="56" t="s">
+      <c r="K13" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="L13" s="64" t="s">
+      <c r="L13" s="41" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B14" s="33"/>
-      <c r="C14" s="61"/>
-      <c r="D14" s="61"/>
-      <c r="E14" s="56" t="s">
+      <c r="B14" s="59"/>
+      <c r="C14" s="54"/>
+      <c r="D14" s="54"/>
+      <c r="E14" s="37" t="s">
         <v>189</v>
       </c>
-      <c r="F14" s="58">
+      <c r="F14" s="36">
         <v>2</v>
       </c>
-      <c r="G14" s="58">
+      <c r="G14" s="36">
         <v>2</v>
       </c>
-      <c r="H14" s="58">
+      <c r="H14" s="36">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="I14" s="58" t="s">
+      <c r="I14" s="36" t="s">
         <v>28</v>
       </c>
-      <c r="J14" s="59" t="s">
+      <c r="J14" s="39" t="s">
         <v>194</v>
       </c>
-      <c r="K14" s="56" t="s">
+      <c r="K14" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="L14" s="64" t="s">
+      <c r="L14" s="41" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B15" s="33"/>
-      <c r="C15" s="61"/>
-      <c r="D15" s="62"/>
-      <c r="E15" s="56" t="s">
+      <c r="B15" s="59"/>
+      <c r="C15" s="54"/>
+      <c r="D15" s="51"/>
+      <c r="E15" s="37" t="s">
         <v>190</v>
       </c>
-      <c r="F15" s="58">
+      <c r="F15" s="36">
         <v>2</v>
       </c>
-      <c r="G15" s="58">
+      <c r="G15" s="36">
         <v>3</v>
       </c>
-      <c r="H15" s="58">
+      <c r="H15" s="36">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="I15" s="58" t="s">
+      <c r="I15" s="36" t="s">
         <v>28</v>
       </c>
-      <c r="J15" s="59" t="s">
+      <c r="J15" s="39" t="s">
         <v>195</v>
       </c>
-      <c r="K15" s="56" t="s">
+      <c r="K15" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="L15" s="64" t="s">
+      <c r="L15" s="41" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B16" s="33"/>
-      <c r="C16" s="61"/>
-      <c r="D16" s="55" t="s">
+      <c r="B16" s="59"/>
+      <c r="C16" s="54"/>
+      <c r="D16" s="50" t="s">
         <v>184</v>
       </c>
-      <c r="E16" s="56" t="s">
+      <c r="E16" s="37" t="s">
         <v>196</v>
       </c>
-      <c r="F16" s="58"/>
-      <c r="G16" s="58"/>
-      <c r="H16" s="58"/>
-      <c r="I16" s="57" t="s">
-        <v>27</v>
-      </c>
-      <c r="J16" s="59"/>
-      <c r="K16" s="56"/>
-      <c r="L16" s="60"/>
+      <c r="F16" s="36"/>
+      <c r="G16" s="36"/>
+      <c r="H16" s="36"/>
+      <c r="I16" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="J16" s="39"/>
+      <c r="K16" s="37"/>
+      <c r="L16" s="40"/>
     </row>
     <row r="17" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B17" s="33"/>
-      <c r="C17" s="61"/>
-      <c r="D17" s="61"/>
-      <c r="E17" s="56" t="s">
+      <c r="B17" s="59"/>
+      <c r="C17" s="54"/>
+      <c r="D17" s="54"/>
+      <c r="E17" s="37" t="s">
         <v>197</v>
       </c>
-      <c r="F17" s="58"/>
-      <c r="G17" s="58"/>
-      <c r="H17" s="58"/>
-      <c r="I17" s="57" t="s">
-        <v>27</v>
-      </c>
-      <c r="J17" s="59"/>
-      <c r="K17" s="56"/>
-      <c r="L17" s="60"/>
+      <c r="F17" s="36"/>
+      <c r="G17" s="36"/>
+      <c r="H17" s="36"/>
+      <c r="I17" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="J17" s="39"/>
+      <c r="K17" s="37"/>
+      <c r="L17" s="40"/>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B18" s="33"/>
-      <c r="C18" s="61"/>
-      <c r="D18" s="61"/>
-      <c r="E18" s="56" t="s">
+      <c r="B18" s="59"/>
+      <c r="C18" s="54"/>
+      <c r="D18" s="54"/>
+      <c r="E18" s="37" t="s">
         <v>198</v>
       </c>
-      <c r="F18" s="58"/>
-      <c r="G18" s="58"/>
-      <c r="H18" s="58"/>
-      <c r="I18" s="57" t="s">
-        <v>27</v>
-      </c>
-      <c r="J18" s="59"/>
-      <c r="K18" s="56"/>
-      <c r="L18" s="60"/>
+      <c r="F18" s="36"/>
+      <c r="G18" s="36"/>
+      <c r="H18" s="36"/>
+      <c r="I18" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="J18" s="39"/>
+      <c r="K18" s="37"/>
+      <c r="L18" s="40"/>
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B19" s="33"/>
-      <c r="C19" s="61"/>
-      <c r="D19" s="61"/>
-      <c r="E19" s="56" t="s">
+      <c r="B19" s="59"/>
+      <c r="C19" s="54"/>
+      <c r="D19" s="54"/>
+      <c r="E19" s="37" t="s">
         <v>199</v>
       </c>
-      <c r="F19" s="58"/>
-      <c r="G19" s="58"/>
-      <c r="H19" s="58"/>
-      <c r="I19" s="57" t="s">
-        <v>27</v>
-      </c>
-      <c r="J19" s="59"/>
-      <c r="K19" s="56"/>
-      <c r="L19" s="60"/>
+      <c r="F19" s="36"/>
+      <c r="G19" s="36"/>
+      <c r="H19" s="36"/>
+      <c r="I19" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="J19" s="39"/>
+      <c r="K19" s="37"/>
+      <c r="L19" s="40"/>
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B20" s="33"/>
-      <c r="C20" s="61"/>
-      <c r="D20" s="62"/>
-      <c r="E20" s="56" t="s">
+      <c r="B20" s="59"/>
+      <c r="C20" s="54"/>
+      <c r="D20" s="51"/>
+      <c r="E20" s="37" t="s">
         <v>200</v>
       </c>
-      <c r="F20" s="58"/>
-      <c r="G20" s="58"/>
-      <c r="H20" s="58"/>
-      <c r="I20" s="57" t="s">
-        <v>27</v>
-      </c>
-      <c r="J20" s="59"/>
-      <c r="K20" s="56"/>
-      <c r="L20" s="60"/>
+      <c r="F20" s="36"/>
+      <c r="G20" s="36"/>
+      <c r="H20" s="36"/>
+      <c r="I20" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="J20" s="39"/>
+      <c r="K20" s="37"/>
+      <c r="L20" s="40"/>
     </row>
     <row r="21" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B21" s="33"/>
-      <c r="C21" s="61"/>
-      <c r="D21" s="61" t="s">
+      <c r="B21" s="59"/>
+      <c r="C21" s="54"/>
+      <c r="D21" s="54" t="s">
         <v>185</v>
       </c>
-      <c r="E21" s="56" t="s">
+      <c r="E21" s="37" t="s">
         <v>201</v>
       </c>
-      <c r="F21" s="58"/>
-      <c r="G21" s="58"/>
-      <c r="H21" s="58"/>
-      <c r="I21" s="57" t="s">
-        <v>27</v>
-      </c>
-      <c r="J21" s="59"/>
-      <c r="K21" s="56"/>
-      <c r="L21" s="60"/>
+      <c r="F21" s="36"/>
+      <c r="G21" s="36"/>
+      <c r="H21" s="36"/>
+      <c r="I21" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="J21" s="39"/>
+      <c r="K21" s="37"/>
+      <c r="L21" s="40"/>
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B22" s="33"/>
-      <c r="C22" s="61"/>
-      <c r="D22" s="61"/>
-      <c r="E22" s="56" t="s">
+      <c r="B22" s="59"/>
+      <c r="C22" s="54"/>
+      <c r="D22" s="54"/>
+      <c r="E22" s="37" t="s">
         <v>213</v>
       </c>
-      <c r="F22" s="58"/>
-      <c r="G22" s="58"/>
-      <c r="H22" s="58"/>
-      <c r="I22" s="57" t="s">
-        <v>27</v>
-      </c>
-      <c r="J22" s="59"/>
-      <c r="K22" s="56"/>
-      <c r="L22" s="60"/>
+      <c r="F22" s="36"/>
+      <c r="G22" s="36"/>
+      <c r="H22" s="36"/>
+      <c r="I22" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="J22" s="39"/>
+      <c r="K22" s="37"/>
+      <c r="L22" s="40"/>
     </row>
     <row r="23" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B23" s="33"/>
-      <c r="C23" s="61"/>
-      <c r="D23" s="61"/>
-      <c r="E23" s="56" t="s">
+      <c r="B23" s="59"/>
+      <c r="C23" s="54"/>
+      <c r="D23" s="54"/>
+      <c r="E23" s="37" t="s">
         <v>202</v>
       </c>
-      <c r="F23" s="58"/>
-      <c r="G23" s="58"/>
-      <c r="H23" s="58"/>
-      <c r="I23" s="57" t="s">
-        <v>27</v>
-      </c>
-      <c r="J23" s="59"/>
-      <c r="K23" s="56"/>
-      <c r="L23" s="60"/>
+      <c r="F23" s="36"/>
+      <c r="G23" s="36"/>
+      <c r="H23" s="36"/>
+      <c r="I23" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="J23" s="39"/>
+      <c r="K23" s="37"/>
+      <c r="L23" s="40"/>
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B24" s="33"/>
-      <c r="C24" s="61"/>
-      <c r="D24" s="61"/>
-      <c r="E24" s="56" t="s">
+      <c r="B24" s="59"/>
+      <c r="C24" s="54"/>
+      <c r="D24" s="54"/>
+      <c r="E24" s="37" t="s">
         <v>203</v>
       </c>
-      <c r="F24" s="58"/>
-      <c r="G24" s="58"/>
-      <c r="H24" s="58"/>
-      <c r="I24" s="57" t="s">
-        <v>27</v>
-      </c>
-      <c r="J24" s="59"/>
-      <c r="K24" s="56"/>
-      <c r="L24" s="60"/>
+      <c r="F24" s="36"/>
+      <c r="G24" s="36"/>
+      <c r="H24" s="36"/>
+      <c r="I24" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="J24" s="39"/>
+      <c r="K24" s="37"/>
+      <c r="L24" s="40"/>
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B25" s="33"/>
-      <c r="C25" s="61"/>
-      <c r="D25" s="61"/>
-      <c r="E25" s="56" t="s">
+      <c r="B25" s="59"/>
+      <c r="C25" s="54"/>
+      <c r="D25" s="54"/>
+      <c r="E25" s="37" t="s">
         <v>204</v>
       </c>
-      <c r="F25" s="58"/>
-      <c r="G25" s="58"/>
-      <c r="H25" s="58"/>
-      <c r="I25" s="57" t="s">
-        <v>27</v>
-      </c>
-      <c r="J25" s="59"/>
-      <c r="K25" s="56"/>
-      <c r="L25" s="60"/>
+      <c r="F25" s="36"/>
+      <c r="G25" s="36"/>
+      <c r="H25" s="36"/>
+      <c r="I25" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="J25" s="39"/>
+      <c r="K25" s="37"/>
+      <c r="L25" s="40"/>
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B26" s="33"/>
-      <c r="C26" s="61"/>
-      <c r="D26" s="61"/>
-      <c r="E26" s="56" t="s">
+      <c r="B26" s="59"/>
+      <c r="C26" s="54"/>
+      <c r="D26" s="54"/>
+      <c r="E26" s="37" t="s">
         <v>205</v>
       </c>
-      <c r="F26" s="58"/>
-      <c r="G26" s="58"/>
-      <c r="H26" s="58"/>
-      <c r="I26" s="57" t="s">
-        <v>27</v>
-      </c>
-      <c r="J26" s="59"/>
-      <c r="K26" s="56"/>
-      <c r="L26" s="60"/>
+      <c r="F26" s="36"/>
+      <c r="G26" s="36"/>
+      <c r="H26" s="36"/>
+      <c r="I26" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="J26" s="39"/>
+      <c r="K26" s="37"/>
+      <c r="L26" s="40"/>
     </row>
     <row r="27" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B27" s="33"/>
-      <c r="C27" s="61"/>
-      <c r="D27" s="61"/>
-      <c r="E27" s="56" t="s">
+      <c r="B27" s="59"/>
+      <c r="C27" s="54"/>
+      <c r="D27" s="54"/>
+      <c r="E27" s="37" t="s">
         <v>214</v>
       </c>
-      <c r="F27" s="58"/>
-      <c r="G27" s="58"/>
-      <c r="H27" s="58"/>
-      <c r="I27" s="57" t="s">
-        <v>27</v>
-      </c>
-      <c r="J27" s="59"/>
-      <c r="K27" s="56"/>
-      <c r="L27" s="60"/>
+      <c r="F27" s="36"/>
+      <c r="G27" s="36"/>
+      <c r="H27" s="36"/>
+      <c r="I27" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="J27" s="39"/>
+      <c r="K27" s="37"/>
+      <c r="L27" s="40"/>
     </row>
     <row r="28" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B28" s="33"/>
-      <c r="C28" s="61"/>
-      <c r="D28" s="61"/>
-      <c r="E28" s="56" t="s">
+      <c r="B28" s="59"/>
+      <c r="C28" s="54"/>
+      <c r="D28" s="54"/>
+      <c r="E28" s="37" t="s">
         <v>206</v>
       </c>
-      <c r="F28" s="58"/>
-      <c r="G28" s="58"/>
-      <c r="H28" s="58"/>
-      <c r="I28" s="57" t="s">
-        <v>27</v>
-      </c>
-      <c r="J28" s="59"/>
-      <c r="K28" s="56"/>
-      <c r="L28" s="60"/>
+      <c r="F28" s="36"/>
+      <c r="G28" s="36"/>
+      <c r="H28" s="36"/>
+      <c r="I28" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="J28" s="39"/>
+      <c r="K28" s="37"/>
+      <c r="L28" s="40"/>
     </row>
     <row r="29" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B29" s="33"/>
-      <c r="C29" s="61"/>
-      <c r="D29" s="61"/>
-      <c r="E29" s="56" t="s">
+      <c r="B29" s="59"/>
+      <c r="C29" s="54"/>
+      <c r="D29" s="54"/>
+      <c r="E29" s="37" t="s">
         <v>207</v>
       </c>
-      <c r="F29" s="58"/>
-      <c r="G29" s="58"/>
-      <c r="H29" s="58"/>
-      <c r="I29" s="57" t="s">
-        <v>27</v>
-      </c>
-      <c r="J29" s="59"/>
-      <c r="K29" s="56"/>
-      <c r="L29" s="60"/>
+      <c r="F29" s="36"/>
+      <c r="G29" s="36"/>
+      <c r="H29" s="36"/>
+      <c r="I29" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="J29" s="39"/>
+      <c r="K29" s="37"/>
+      <c r="L29" s="40"/>
     </row>
     <row r="30" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B30" s="33"/>
-      <c r="C30" s="61"/>
-      <c r="D30" s="61"/>
-      <c r="E30" s="56" t="s">
+      <c r="B30" s="59"/>
+      <c r="C30" s="54"/>
+      <c r="D30" s="54"/>
+      <c r="E30" s="37" t="s">
         <v>208</v>
       </c>
-      <c r="F30" s="58"/>
-      <c r="G30" s="58"/>
-      <c r="H30" s="58"/>
-      <c r="I30" s="57" t="s">
-        <v>27</v>
-      </c>
-      <c r="J30" s="59"/>
-      <c r="K30" s="56"/>
-      <c r="L30" s="60"/>
+      <c r="F30" s="36"/>
+      <c r="G30" s="36"/>
+      <c r="H30" s="36"/>
+      <c r="I30" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="J30" s="39"/>
+      <c r="K30" s="37"/>
+      <c r="L30" s="40"/>
     </row>
     <row r="31" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B31" s="33"/>
-      <c r="C31" s="61"/>
-      <c r="D31" s="61"/>
-      <c r="E31" s="56" t="s">
+      <c r="B31" s="59"/>
+      <c r="C31" s="54"/>
+      <c r="D31" s="54"/>
+      <c r="E31" s="37" t="s">
         <v>209</v>
       </c>
-      <c r="F31" s="58"/>
-      <c r="G31" s="58"/>
-      <c r="H31" s="58"/>
-      <c r="I31" s="57" t="s">
-        <v>27</v>
-      </c>
-      <c r="J31" s="59"/>
-      <c r="K31" s="56"/>
-      <c r="L31" s="60"/>
+      <c r="F31" s="36"/>
+      <c r="G31" s="36"/>
+      <c r="H31" s="36"/>
+      <c r="I31" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="J31" s="39"/>
+      <c r="K31" s="37"/>
+      <c r="L31" s="40"/>
     </row>
     <row r="32" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B32" s="33"/>
-      <c r="C32" s="61"/>
-      <c r="D32" s="61"/>
-      <c r="E32" s="56" t="s">
+      <c r="B32" s="59"/>
+      <c r="C32" s="54"/>
+      <c r="D32" s="54"/>
+      <c r="E32" s="37" t="s">
         <v>210</v>
       </c>
-      <c r="F32" s="58"/>
-      <c r="G32" s="58"/>
-      <c r="H32" s="58"/>
-      <c r="I32" s="57" t="s">
-        <v>27</v>
-      </c>
-      <c r="J32" s="59"/>
-      <c r="K32" s="56"/>
-      <c r="L32" s="60"/>
+      <c r="F32" s="36"/>
+      <c r="G32" s="36"/>
+      <c r="H32" s="36"/>
+      <c r="I32" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="J32" s="39"/>
+      <c r="K32" s="37"/>
+      <c r="L32" s="40"/>
     </row>
     <row r="33" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B33" s="33"/>
-      <c r="C33" s="61"/>
-      <c r="D33" s="61"/>
-      <c r="E33" s="56" t="s">
+      <c r="B33" s="59"/>
+      <c r="C33" s="54"/>
+      <c r="D33" s="54"/>
+      <c r="E33" s="37" t="s">
         <v>211</v>
       </c>
-      <c r="F33" s="58"/>
-      <c r="G33" s="58"/>
-      <c r="H33" s="58"/>
-      <c r="I33" s="57" t="s">
-        <v>27</v>
-      </c>
-      <c r="J33" s="59"/>
-      <c r="K33" s="56"/>
-      <c r="L33" s="60"/>
+      <c r="F33" s="36"/>
+      <c r="G33" s="36"/>
+      <c r="H33" s="36"/>
+      <c r="I33" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="J33" s="39"/>
+      <c r="K33" s="37"/>
+      <c r="L33" s="40"/>
     </row>
     <row r="34" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B34" s="33"/>
-      <c r="C34" s="62"/>
-      <c r="D34" s="62"/>
-      <c r="E34" s="56" t="s">
+      <c r="B34" s="59"/>
+      <c r="C34" s="51"/>
+      <c r="D34" s="51"/>
+      <c r="E34" s="37" t="s">
         <v>212</v>
       </c>
-      <c r="F34" s="58"/>
-      <c r="G34" s="58"/>
-      <c r="H34" s="58"/>
-      <c r="I34" s="57" t="s">
-        <v>27</v>
-      </c>
-      <c r="J34" s="59"/>
-      <c r="K34" s="56"/>
-      <c r="L34" s="60"/>
+      <c r="F34" s="36"/>
+      <c r="G34" s="36"/>
+      <c r="H34" s="36"/>
+      <c r="I34" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="J34" s="39"/>
+      <c r="K34" s="37"/>
+      <c r="L34" s="40"/>
     </row>
     <row r="35" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B35" s="33"/>
-      <c r="C35" s="31" t="s">
+      <c r="B35" s="59"/>
+      <c r="C35" s="61" t="s">
         <v>105</v>
       </c>
-      <c r="D35" s="38" t="s">
+      <c r="D35" s="56" t="s">
         <v>100</v>
       </c>
       <c r="E35" s="7" t="s">
@@ -2837,7 +2834,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I35" s="37" t="s">
+      <c r="I35" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J35" s="6"/>
@@ -2845,9 +2842,9 @@
       <c r="L35" s="7"/>
     </row>
     <row r="36" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B36" s="33"/>
-      <c r="C36" s="31"/>
-      <c r="D36" s="40"/>
+      <c r="B36" s="59"/>
+      <c r="C36" s="61"/>
+      <c r="D36" s="57"/>
       <c r="E36" s="7" t="s">
         <v>102</v>
       </c>
@@ -2857,7 +2854,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I36" s="37" t="s">
+      <c r="I36" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J36" s="6"/>
@@ -2865,9 +2862,9 @@
       <c r="L36" s="7"/>
     </row>
     <row r="37" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B37" s="33"/>
-      <c r="C37" s="31"/>
-      <c r="D37" s="40"/>
+      <c r="B37" s="59"/>
+      <c r="C37" s="61"/>
+      <c r="D37" s="57"/>
       <c r="E37" s="7" t="s">
         <v>103</v>
       </c>
@@ -2877,7 +2874,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I37" s="37" t="s">
+      <c r="I37" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J37" s="6"/>
@@ -2885,9 +2882,9 @@
       <c r="L37" s="7"/>
     </row>
     <row r="38" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B38" s="33"/>
-      <c r="C38" s="31"/>
-      <c r="D38" s="42"/>
+      <c r="B38" s="59"/>
+      <c r="C38" s="61"/>
+      <c r="D38" s="58"/>
       <c r="E38" s="7" t="s">
         <v>104</v>
       </c>
@@ -2897,7 +2894,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I38" s="37" t="s">
+      <c r="I38" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J38" s="6"/>
@@ -2905,9 +2902,9 @@
       <c r="L38" s="7"/>
     </row>
     <row r="39" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B39" s="33"/>
-      <c r="C39" s="31"/>
-      <c r="D39" s="34" t="s">
+      <c r="B39" s="59"/>
+      <c r="C39" s="61"/>
+      <c r="D39" s="52" t="s">
         <v>106</v>
       </c>
       <c r="E39" s="7" t="s">
@@ -2919,7 +2916,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I39" s="37" t="s">
+      <c r="I39" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J39" s="6"/>
@@ -2927,9 +2924,9 @@
       <c r="L39" s="7"/>
     </row>
     <row r="40" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B40" s="33"/>
-      <c r="C40" s="31"/>
-      <c r="D40" s="35"/>
+      <c r="B40" s="59"/>
+      <c r="C40" s="61"/>
+      <c r="D40" s="55"/>
       <c r="E40" s="7" t="s">
         <v>107</v>
       </c>
@@ -2939,7 +2936,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I40" s="37" t="s">
+      <c r="I40" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J40" s="6"/>
@@ -2947,9 +2944,9 @@
       <c r="L40" s="7"/>
     </row>
     <row r="41" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B41" s="33"/>
-      <c r="C41" s="31"/>
-      <c r="D41" s="35"/>
+      <c r="B41" s="59"/>
+      <c r="C41" s="61"/>
+      <c r="D41" s="55"/>
       <c r="E41" s="7" t="s">
         <v>108</v>
       </c>
@@ -2959,7 +2956,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I41" s="37" t="s">
+      <c r="I41" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J41" s="6"/>
@@ -2967,9 +2964,9 @@
       <c r="L41" s="7"/>
     </row>
     <row r="42" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B42" s="33"/>
-      <c r="C42" s="31"/>
-      <c r="D42" s="35"/>
+      <c r="B42" s="59"/>
+      <c r="C42" s="61"/>
+      <c r="D42" s="55"/>
       <c r="E42" s="7" t="s">
         <v>109</v>
       </c>
@@ -2979,7 +2976,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I42" s="37" t="s">
+      <c r="I42" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J42" s="6"/>
@@ -2987,9 +2984,9 @@
       <c r="L42" s="7"/>
     </row>
     <row r="43" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B43" s="33"/>
-      <c r="C43" s="31"/>
-      <c r="D43" s="35"/>
+      <c r="B43" s="59"/>
+      <c r="C43" s="61"/>
+      <c r="D43" s="55"/>
       <c r="E43" s="7" t="s">
         <v>153</v>
       </c>
@@ -2999,7 +2996,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I43" s="37" t="s">
+      <c r="I43" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J43" s="6"/>
@@ -3007,9 +3004,9 @@
       <c r="L43" s="7"/>
     </row>
     <row r="44" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B44" s="33"/>
-      <c r="C44" s="31"/>
-      <c r="D44" s="35"/>
+      <c r="B44" s="59"/>
+      <c r="C44" s="61"/>
+      <c r="D44" s="55"/>
       <c r="E44" s="7" t="s">
         <v>110</v>
       </c>
@@ -3019,7 +3016,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I44" s="37" t="s">
+      <c r="I44" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J44" s="6"/>
@@ -3027,9 +3024,9 @@
       <c r="L44" s="7"/>
     </row>
     <row r="45" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B45" s="33"/>
-      <c r="C45" s="31"/>
-      <c r="D45" s="35"/>
+      <c r="B45" s="59"/>
+      <c r="C45" s="61"/>
+      <c r="D45" s="55"/>
       <c r="E45" s="7" t="s">
         <v>111</v>
       </c>
@@ -3039,7 +3036,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I45" s="37" t="s">
+      <c r="I45" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J45" s="6"/>
@@ -3047,9 +3044,9 @@
       <c r="L45" s="7"/>
     </row>
     <row r="46" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B46" s="33"/>
-      <c r="C46" s="31"/>
-      <c r="D46" s="35"/>
+      <c r="B46" s="59"/>
+      <c r="C46" s="61"/>
+      <c r="D46" s="55"/>
       <c r="E46" s="7" t="s">
         <v>112</v>
       </c>
@@ -3059,7 +3056,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I46" s="37" t="s">
+      <c r="I46" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J46" s="6"/>
@@ -3067,9 +3064,9 @@
       <c r="L46" s="7"/>
     </row>
     <row r="47" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B47" s="33"/>
-      <c r="C47" s="31"/>
-      <c r="D47" s="35"/>
+      <c r="B47" s="59"/>
+      <c r="C47" s="61"/>
+      <c r="D47" s="55"/>
       <c r="E47" s="7" t="s">
         <v>154</v>
       </c>
@@ -3079,7 +3076,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I47" s="37" t="s">
+      <c r="I47" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J47" s="6"/>
@@ -3087,9 +3084,9 @@
       <c r="L47" s="7"/>
     </row>
     <row r="48" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B48" s="33"/>
-      <c r="C48" s="31"/>
-      <c r="D48" s="35"/>
+      <c r="B48" s="59"/>
+      <c r="C48" s="61"/>
+      <c r="D48" s="55"/>
       <c r="E48" s="7" t="s">
         <v>113</v>
       </c>
@@ -3099,7 +3096,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I48" s="37" t="s">
+      <c r="I48" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J48" s="6"/>
@@ -3107,9 +3104,9 @@
       <c r="L48" s="7"/>
     </row>
     <row r="49" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B49" s="33"/>
-      <c r="C49" s="31"/>
-      <c r="D49" s="35"/>
+      <c r="B49" s="59"/>
+      <c r="C49" s="61"/>
+      <c r="D49" s="55"/>
       <c r="E49" s="7" t="s">
         <v>114</v>
       </c>
@@ -3119,7 +3116,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I49" s="37" t="s">
+      <c r="I49" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J49" s="6"/>
@@ -3127,9 +3124,9 @@
       <c r="L49" s="7"/>
     </row>
     <row r="50" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B50" s="33"/>
-      <c r="C50" s="31"/>
-      <c r="D50" s="35"/>
+      <c r="B50" s="59"/>
+      <c r="C50" s="61"/>
+      <c r="D50" s="55"/>
       <c r="E50" s="7" t="s">
         <v>115</v>
       </c>
@@ -3139,7 +3136,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I50" s="37" t="s">
+      <c r="I50" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J50" s="6"/>
@@ -3147,9 +3144,9 @@
       <c r="L50" s="7"/>
     </row>
     <row r="51" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B51" s="33"/>
-      <c r="C51" s="31"/>
-      <c r="D51" s="35"/>
+      <c r="B51" s="59"/>
+      <c r="C51" s="61"/>
+      <c r="D51" s="55"/>
       <c r="E51" s="7" t="s">
         <v>155</v>
       </c>
@@ -3159,7 +3156,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I51" s="37" t="s">
+      <c r="I51" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J51" s="6"/>
@@ -3167,9 +3164,9 @@
       <c r="L51" s="7"/>
     </row>
     <row r="52" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B52" s="33"/>
-      <c r="C52" s="31"/>
-      <c r="D52" s="35"/>
+      <c r="B52" s="59"/>
+      <c r="C52" s="61"/>
+      <c r="D52" s="55"/>
       <c r="E52" s="7" t="s">
         <v>116</v>
       </c>
@@ -3179,7 +3176,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I52" s="37" t="s">
+      <c r="I52" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J52" s="6"/>
@@ -3187,9 +3184,9 @@
       <c r="L52" s="7"/>
     </row>
     <row r="53" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B53" s="33"/>
-      <c r="C53" s="31"/>
-      <c r="D53" s="35"/>
+      <c r="B53" s="59"/>
+      <c r="C53" s="61"/>
+      <c r="D53" s="55"/>
       <c r="E53" s="7" t="s">
         <v>117</v>
       </c>
@@ -3199,7 +3196,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I53" s="37" t="s">
+      <c r="I53" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J53" s="6"/>
@@ -3207,9 +3204,9 @@
       <c r="L53" s="7"/>
     </row>
     <row r="54" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B54" s="33"/>
-      <c r="C54" s="31"/>
-      <c r="D54" s="35"/>
+      <c r="B54" s="59"/>
+      <c r="C54" s="61"/>
+      <c r="D54" s="55"/>
       <c r="E54" s="7" t="s">
         <v>118</v>
       </c>
@@ -3219,7 +3216,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I54" s="37" t="s">
+      <c r="I54" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J54" s="6"/>
@@ -3227,9 +3224,9 @@
       <c r="L54" s="7"/>
     </row>
     <row r="55" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B55" s="33"/>
-      <c r="C55" s="31"/>
-      <c r="D55" s="35"/>
+      <c r="B55" s="59"/>
+      <c r="C55" s="61"/>
+      <c r="D55" s="55"/>
       <c r="E55" s="7" t="s">
         <v>156</v>
       </c>
@@ -3239,7 +3236,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I55" s="37" t="s">
+      <c r="I55" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J55" s="6"/>
@@ -3247,9 +3244,9 @@
       <c r="L55" s="7"/>
     </row>
     <row r="56" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B56" s="33"/>
-      <c r="C56" s="31"/>
-      <c r="D56" s="35"/>
+      <c r="B56" s="59"/>
+      <c r="C56" s="61"/>
+      <c r="D56" s="55"/>
       <c r="E56" s="7" t="s">
         <v>119</v>
       </c>
@@ -3259,7 +3256,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I56" s="37" t="s">
+      <c r="I56" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J56" s="6"/>
@@ -3267,9 +3264,9 @@
       <c r="L56" s="7"/>
     </row>
     <row r="57" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B57" s="33"/>
-      <c r="C57" s="31"/>
-      <c r="D57" s="35"/>
+      <c r="B57" s="59"/>
+      <c r="C57" s="61"/>
+      <c r="D57" s="55"/>
       <c r="E57" s="7" t="s">
         <v>120</v>
       </c>
@@ -3279,7 +3276,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I57" s="37" t="s">
+      <c r="I57" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J57" s="6"/>
@@ -3287,9 +3284,9 @@
       <c r="L57" s="7"/>
     </row>
     <row r="58" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B58" s="33"/>
-      <c r="C58" s="31"/>
-      <c r="D58" s="36"/>
+      <c r="B58" s="59"/>
+      <c r="C58" s="61"/>
+      <c r="D58" s="53"/>
       <c r="E58" s="7" t="s">
         <v>121</v>
       </c>
@@ -3299,7 +3296,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I58" s="37" t="s">
+      <c r="I58" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J58" s="6"/>
@@ -3307,9 +3304,9 @@
       <c r="L58" s="7"/>
     </row>
     <row r="59" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B59" s="33"/>
-      <c r="C59" s="31"/>
-      <c r="D59" s="34" t="s">
+      <c r="B59" s="59"/>
+      <c r="C59" s="61"/>
+      <c r="D59" s="52" t="s">
         <v>133</v>
       </c>
       <c r="E59" s="7" t="s">
@@ -3321,7 +3318,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I59" s="37" t="s">
+      <c r="I59" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J59" s="6"/>
@@ -3329,9 +3326,9 @@
       <c r="L59" s="7"/>
     </row>
     <row r="60" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B60" s="33"/>
-      <c r="C60" s="31"/>
-      <c r="D60" s="35"/>
+      <c r="B60" s="59"/>
+      <c r="C60" s="61"/>
+      <c r="D60" s="55"/>
       <c r="E60" s="7" t="s">
         <v>134</v>
       </c>
@@ -3341,7 +3338,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I60" s="37" t="s">
+      <c r="I60" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J60" s="6"/>
@@ -3349,9 +3346,9 @@
       <c r="L60" s="7"/>
     </row>
     <row r="61" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B61" s="33"/>
-      <c r="C61" s="31"/>
-      <c r="D61" s="35"/>
+      <c r="B61" s="59"/>
+      <c r="C61" s="61"/>
+      <c r="D61" s="55"/>
       <c r="E61" s="7" t="s">
         <v>135</v>
       </c>
@@ -3361,7 +3358,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I61" s="37" t="s">
+      <c r="I61" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J61" s="6"/>
@@ -3369,9 +3366,9 @@
       <c r="L61" s="7"/>
     </row>
     <row r="62" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B62" s="33"/>
-      <c r="C62" s="31"/>
-      <c r="D62" s="35"/>
+      <c r="B62" s="59"/>
+      <c r="C62" s="61"/>
+      <c r="D62" s="55"/>
       <c r="E62" s="7" t="s">
         <v>136</v>
       </c>
@@ -3381,7 +3378,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I62" s="37" t="s">
+      <c r="I62" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J62" s="6"/>
@@ -3389,9 +3386,9 @@
       <c r="L62" s="7"/>
     </row>
     <row r="63" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B63" s="33"/>
-      <c r="C63" s="31"/>
-      <c r="D63" s="35"/>
+      <c r="B63" s="59"/>
+      <c r="C63" s="61"/>
+      <c r="D63" s="55"/>
       <c r="E63" s="7" t="s">
         <v>137</v>
       </c>
@@ -3401,7 +3398,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I63" s="37" t="s">
+      <c r="I63" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J63" s="6"/>
@@ -3409,9 +3406,9 @@
       <c r="L63" s="7"/>
     </row>
     <row r="64" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B64" s="33"/>
-      <c r="C64" s="31"/>
-      <c r="D64" s="35"/>
+      <c r="B64" s="59"/>
+      <c r="C64" s="61"/>
+      <c r="D64" s="55"/>
       <c r="E64" s="7" t="s">
         <v>138</v>
       </c>
@@ -3421,7 +3418,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I64" s="37" t="s">
+      <c r="I64" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J64" s="6"/>
@@ -3429,9 +3426,9 @@
       <c r="L64" s="7"/>
     </row>
     <row r="65" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B65" s="33"/>
-      <c r="C65" s="31"/>
-      <c r="D65" s="35"/>
+      <c r="B65" s="59"/>
+      <c r="C65" s="61"/>
+      <c r="D65" s="55"/>
       <c r="E65" s="7" t="s">
         <v>158</v>
       </c>
@@ -3441,7 +3438,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I65" s="37" t="s">
+      <c r="I65" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J65" s="6"/>
@@ -3449,9 +3446,9 @@
       <c r="L65" s="7"/>
     </row>
     <row r="66" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B66" s="33"/>
-      <c r="C66" s="31"/>
-      <c r="D66" s="35"/>
+      <c r="B66" s="59"/>
+      <c r="C66" s="61"/>
+      <c r="D66" s="55"/>
       <c r="E66" s="7" t="s">
         <v>140</v>
       </c>
@@ -3461,7 +3458,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I66" s="37" t="s">
+      <c r="I66" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J66" s="6"/>
@@ -3469,9 +3466,9 @@
       <c r="L66" s="7"/>
     </row>
     <row r="67" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B67" s="33"/>
-      <c r="C67" s="31"/>
-      <c r="D67" s="35"/>
+      <c r="B67" s="59"/>
+      <c r="C67" s="61"/>
+      <c r="D67" s="55"/>
       <c r="E67" s="7" t="s">
         <v>141</v>
       </c>
@@ -3481,7 +3478,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I67" s="37" t="s">
+      <c r="I67" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J67" s="6"/>
@@ -3489,9 +3486,9 @@
       <c r="L67" s="7"/>
     </row>
     <row r="68" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B68" s="33"/>
-      <c r="C68" s="31"/>
-      <c r="D68" s="35"/>
+      <c r="B68" s="59"/>
+      <c r="C68" s="61"/>
+      <c r="D68" s="55"/>
       <c r="E68" s="7" t="s">
         <v>142</v>
       </c>
@@ -3501,7 +3498,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I68" s="37" t="s">
+      <c r="I68" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J68" s="6"/>
@@ -3509,9 +3506,9 @@
       <c r="L68" s="7"/>
     </row>
     <row r="69" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B69" s="33"/>
-      <c r="C69" s="31"/>
-      <c r="D69" s="35"/>
+      <c r="B69" s="59"/>
+      <c r="C69" s="61"/>
+      <c r="D69" s="55"/>
       <c r="E69" s="7" t="s">
         <v>139</v>
       </c>
@@ -3521,7 +3518,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I69" s="37" t="s">
+      <c r="I69" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J69" s="6"/>
@@ -3529,9 +3526,9 @@
       <c r="L69" s="7"/>
     </row>
     <row r="70" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B70" s="33"/>
-      <c r="C70" s="31"/>
-      <c r="D70" s="34" t="s">
+      <c r="B70" s="59"/>
+      <c r="C70" s="61"/>
+      <c r="D70" s="52" t="s">
         <v>143</v>
       </c>
       <c r="E70" s="7" t="s">
@@ -3543,7 +3540,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I70" s="37" t="s">
+      <c r="I70" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J70" s="6"/>
@@ -3551,9 +3548,9 @@
       <c r="L70" s="7"/>
     </row>
     <row r="71" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B71" s="33"/>
-      <c r="C71" s="31"/>
-      <c r="D71" s="35"/>
+      <c r="B71" s="59"/>
+      <c r="C71" s="61"/>
+      <c r="D71" s="55"/>
       <c r="E71" s="7" t="s">
         <v>144</v>
       </c>
@@ -3563,7 +3560,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I71" s="37" t="s">
+      <c r="I71" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J71" s="6"/>
@@ -3571,9 +3568,9 @@
       <c r="L71" s="7"/>
     </row>
     <row r="72" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B72" s="33"/>
-      <c r="C72" s="31"/>
-      <c r="D72" s="35"/>
+      <c r="B72" s="59"/>
+      <c r="C72" s="61"/>
+      <c r="D72" s="55"/>
       <c r="E72" s="7" t="s">
         <v>145</v>
       </c>
@@ -3583,7 +3580,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I72" s="37" t="s">
+      <c r="I72" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J72" s="6"/>
@@ -3591,9 +3588,9 @@
       <c r="L72" s="7"/>
     </row>
     <row r="73" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B73" s="33"/>
-      <c r="C73" s="31"/>
-      <c r="D73" s="35"/>
+      <c r="B73" s="59"/>
+      <c r="C73" s="61"/>
+      <c r="D73" s="55"/>
       <c r="E73" s="7" t="s">
         <v>146</v>
       </c>
@@ -3603,7 +3600,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I73" s="37" t="s">
+      <c r="I73" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J73" s="6"/>
@@ -3611,9 +3608,9 @@
       <c r="L73" s="7"/>
     </row>
     <row r="74" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B74" s="33"/>
-      <c r="C74" s="31"/>
-      <c r="D74" s="35"/>
+      <c r="B74" s="59"/>
+      <c r="C74" s="61"/>
+      <c r="D74" s="55"/>
       <c r="E74" s="7" t="s">
         <v>160</v>
       </c>
@@ -3623,7 +3620,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I74" s="37" t="s">
+      <c r="I74" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J74" s="6"/>
@@ -3631,9 +3628,9 @@
       <c r="L74" s="7"/>
     </row>
     <row r="75" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B75" s="33"/>
-      <c r="C75" s="31"/>
-      <c r="D75" s="35"/>
+      <c r="B75" s="59"/>
+      <c r="C75" s="61"/>
+      <c r="D75" s="55"/>
       <c r="E75" s="7" t="s">
         <v>147</v>
       </c>
@@ -3643,7 +3640,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I75" s="37" t="s">
+      <c r="I75" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J75" s="6"/>
@@ -3651,9 +3648,9 @@
       <c r="L75" s="7"/>
     </row>
     <row r="76" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B76" s="33"/>
-      <c r="C76" s="31"/>
-      <c r="D76" s="35"/>
+      <c r="B76" s="59"/>
+      <c r="C76" s="61"/>
+      <c r="D76" s="55"/>
       <c r="E76" s="7" t="s">
         <v>148</v>
       </c>
@@ -3663,7 +3660,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I76" s="37" t="s">
+      <c r="I76" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J76" s="6"/>
@@ -3671,9 +3668,9 @@
       <c r="L76" s="7"/>
     </row>
     <row r="77" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B77" s="33"/>
-      <c r="C77" s="31"/>
-      <c r="D77" s="35"/>
+      <c r="B77" s="59"/>
+      <c r="C77" s="61"/>
+      <c r="D77" s="55"/>
       <c r="E77" s="7" t="s">
         <v>147</v>
       </c>
@@ -3683,7 +3680,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I77" s="37" t="s">
+      <c r="I77" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J77" s="6"/>
@@ -3691,9 +3688,9 @@
       <c r="L77" s="7"/>
     </row>
     <row r="78" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B78" s="33"/>
-      <c r="C78" s="31"/>
-      <c r="D78" s="35"/>
+      <c r="B78" s="59"/>
+      <c r="C78" s="61"/>
+      <c r="D78" s="55"/>
       <c r="E78" s="7" t="s">
         <v>161</v>
       </c>
@@ -3703,7 +3700,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I78" s="37" t="s">
+      <c r="I78" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J78" s="6"/>
@@ -3711,9 +3708,9 @@
       <c r="L78" s="7"/>
     </row>
     <row r="79" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B79" s="33"/>
-      <c r="C79" s="31"/>
-      <c r="D79" s="35"/>
+      <c r="B79" s="59"/>
+      <c r="C79" s="61"/>
+      <c r="D79" s="55"/>
       <c r="E79" s="7" t="s">
         <v>149</v>
       </c>
@@ -3723,7 +3720,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I79" s="37" t="s">
+      <c r="I79" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J79" s="6"/>
@@ -3731,9 +3728,9 @@
       <c r="L79" s="7"/>
     </row>
     <row r="80" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B80" s="33"/>
-      <c r="C80" s="31"/>
-      <c r="D80" s="35"/>
+      <c r="B80" s="59"/>
+      <c r="C80" s="61"/>
+      <c r="D80" s="55"/>
       <c r="E80" s="7" t="s">
         <v>150</v>
       </c>
@@ -3743,7 +3740,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I80" s="37" t="s">
+      <c r="I80" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J80" s="6"/>
@@ -3751,9 +3748,9 @@
       <c r="L80" s="7"/>
     </row>
     <row r="81" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B81" s="33"/>
-      <c r="C81" s="31"/>
-      <c r="D81" s="35"/>
+      <c r="B81" s="59"/>
+      <c r="C81" s="61"/>
+      <c r="D81" s="55"/>
       <c r="E81" s="7" t="s">
         <v>151</v>
       </c>
@@ -3763,7 +3760,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I81" s="37" t="s">
+      <c r="I81" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J81" s="6"/>
@@ -3771,9 +3768,9 @@
       <c r="L81" s="7"/>
     </row>
     <row r="82" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B82" s="33"/>
-      <c r="C82" s="31"/>
-      <c r="D82" s="35"/>
+      <c r="B82" s="59"/>
+      <c r="C82" s="61"/>
+      <c r="D82" s="55"/>
       <c r="E82" s="7" t="s">
         <v>162</v>
       </c>
@@ -3783,7 +3780,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I82" s="37" t="s">
+      <c r="I82" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J82" s="6"/>
@@ -3791,9 +3788,9 @@
       <c r="L82" s="7"/>
     </row>
     <row r="83" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B83" s="33"/>
-      <c r="C83" s="31"/>
-      <c r="D83" s="35"/>
+      <c r="B83" s="59"/>
+      <c r="C83" s="61"/>
+      <c r="D83" s="55"/>
       <c r="E83" s="7" t="s">
         <v>163</v>
       </c>
@@ -3803,7 +3800,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I83" s="37" t="s">
+      <c r="I83" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J83" s="6"/>
@@ -3811,9 +3808,9 @@
       <c r="L83" s="7"/>
     </row>
     <row r="84" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B84" s="33"/>
-      <c r="C84" s="31"/>
-      <c r="D84" s="35"/>
+      <c r="B84" s="59"/>
+      <c r="C84" s="61"/>
+      <c r="D84" s="55"/>
       <c r="E84" s="7" t="s">
         <v>164</v>
       </c>
@@ -3823,7 +3820,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I84" s="37" t="s">
+      <c r="I84" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J84" s="6"/>
@@ -3831,9 +3828,9 @@
       <c r="L84" s="7"/>
     </row>
     <row r="85" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B85" s="33"/>
-      <c r="C85" s="31"/>
-      <c r="D85" s="35"/>
+      <c r="B85" s="59"/>
+      <c r="C85" s="61"/>
+      <c r="D85" s="55"/>
       <c r="E85" s="7" t="s">
         <v>165</v>
       </c>
@@ -3843,7 +3840,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I85" s="37" t="s">
+      <c r="I85" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J85" s="6"/>
@@ -3851,9 +3848,9 @@
       <c r="L85" s="7"/>
     </row>
     <row r="86" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B86" s="33"/>
-      <c r="C86" s="31"/>
-      <c r="D86" s="35"/>
+      <c r="B86" s="59"/>
+      <c r="C86" s="61"/>
+      <c r="D86" s="55"/>
       <c r="E86" s="7" t="s">
         <v>166</v>
       </c>
@@ -3863,7 +3860,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I86" s="37" t="s">
+      <c r="I86" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J86" s="6"/>
@@ -3871,9 +3868,9 @@
       <c r="L86" s="7"/>
     </row>
     <row r="87" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B87" s="33"/>
-      <c r="C87" s="31"/>
-      <c r="D87" s="35"/>
+      <c r="B87" s="59"/>
+      <c r="C87" s="61"/>
+      <c r="D87" s="55"/>
       <c r="E87" s="7" t="s">
         <v>167</v>
       </c>
@@ -3883,7 +3880,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I87" s="37" t="s">
+      <c r="I87" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J87" s="6"/>
@@ -3891,9 +3888,9 @@
       <c r="L87" s="7"/>
     </row>
     <row r="88" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B88" s="33"/>
-      <c r="C88" s="31"/>
-      <c r="D88" s="35"/>
+      <c r="B88" s="59"/>
+      <c r="C88" s="61"/>
+      <c r="D88" s="55"/>
       <c r="E88" s="7" t="s">
         <v>168</v>
       </c>
@@ -3903,7 +3900,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I88" s="37" t="s">
+      <c r="I88" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J88" s="6"/>
@@ -3911,9 +3908,9 @@
       <c r="L88" s="7"/>
     </row>
     <row r="89" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B89" s="33"/>
-      <c r="C89" s="31"/>
-      <c r="D89" s="35"/>
+      <c r="B89" s="59"/>
+      <c r="C89" s="61"/>
+      <c r="D89" s="55"/>
       <c r="E89" s="7" t="s">
         <v>169</v>
       </c>
@@ -3923,7 +3920,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I89" s="37" t="s">
+      <c r="I89" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J89" s="6"/>
@@ -3931,12 +3928,12 @@
       <c r="L89" s="7"/>
     </row>
     <row r="90" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B90" s="33"/>
-      <c r="C90" s="31"/>
-      <c r="D90" s="39" t="s">
+      <c r="B90" s="59"/>
+      <c r="C90" s="61"/>
+      <c r="D90" s="62" t="s">
         <v>170</v>
       </c>
-      <c r="E90" s="63" t="s">
+      <c r="E90" s="42" t="s">
         <v>174</v>
       </c>
       <c r="F90" s="7"/>
@@ -3945,7 +3942,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I90" s="37" t="s">
+      <c r="I90" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J90" s="6"/>
@@ -3953,10 +3950,10 @@
       <c r="L90" s="7"/>
     </row>
     <row r="91" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B91" s="33"/>
-      <c r="C91" s="31"/>
-      <c r="D91" s="41"/>
-      <c r="E91" s="63" t="s">
+      <c r="B91" s="59"/>
+      <c r="C91" s="61"/>
+      <c r="D91" s="63"/>
+      <c r="E91" s="42" t="s">
         <v>171</v>
       </c>
       <c r="F91" s="7"/>
@@ -3965,7 +3962,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I91" s="37" t="s">
+      <c r="I91" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J91" s="6"/>
@@ -3973,10 +3970,10 @@
       <c r="L91" s="7"/>
     </row>
     <row r="92" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B92" s="33"/>
-      <c r="C92" s="31"/>
-      <c r="D92" s="41"/>
-      <c r="E92" s="63" t="s">
+      <c r="B92" s="59"/>
+      <c r="C92" s="61"/>
+      <c r="D92" s="63"/>
+      <c r="E92" s="42" t="s">
         <v>172</v>
       </c>
       <c r="F92" s="7"/>
@@ -3985,7 +3982,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I92" s="37" t="s">
+      <c r="I92" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J92" s="6"/>
@@ -3993,10 +3990,10 @@
       <c r="L92" s="7"/>
     </row>
     <row r="93" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B93" s="33"/>
-      <c r="C93" s="31"/>
-      <c r="D93" s="43"/>
-      <c r="E93" s="63" t="s">
+      <c r="B93" s="59"/>
+      <c r="C93" s="61"/>
+      <c r="D93" s="64"/>
+      <c r="E93" s="42" t="s">
         <v>173</v>
       </c>
       <c r="F93" s="7"/>
@@ -4005,7 +4002,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I93" s="37" t="s">
+      <c r="I93" s="26" t="s">
         <v>27</v>
       </c>
       <c r="J93" s="6"/>
@@ -4014,6 +4011,26 @@
     </row>
   </sheetData>
   <mergeCells count="29">
+    <mergeCell ref="B2:B93"/>
+    <mergeCell ref="C2:C9"/>
+    <mergeCell ref="C35:C93"/>
+    <mergeCell ref="D70:D89"/>
+    <mergeCell ref="D90:D93"/>
+    <mergeCell ref="D35:D38"/>
+    <mergeCell ref="D39:D58"/>
+    <mergeCell ref="D59:D69"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="G5:G6"/>
+    <mergeCell ref="H5:H6"/>
+    <mergeCell ref="C10:C34"/>
+    <mergeCell ref="D21:D34"/>
+    <mergeCell ref="D16:D20"/>
+    <mergeCell ref="D10:D15"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="D2:D6"/>
+    <mergeCell ref="D7:D9"/>
     <mergeCell ref="H12:H13"/>
     <mergeCell ref="I5:I6"/>
     <mergeCell ref="I2:I3"/>
@@ -4021,59 +4038,39 @@
     <mergeCell ref="E12:E13"/>
     <mergeCell ref="F12:F13"/>
     <mergeCell ref="G12:G13"/>
-    <mergeCell ref="C10:C34"/>
-    <mergeCell ref="D21:D34"/>
-    <mergeCell ref="D16:D20"/>
-    <mergeCell ref="D10:D15"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="E5:E6"/>
     <mergeCell ref="F2:F3"/>
     <mergeCell ref="F5:F6"/>
-    <mergeCell ref="D2:D6"/>
-    <mergeCell ref="D7:D9"/>
-    <mergeCell ref="D35:D38"/>
-    <mergeCell ref="D39:D58"/>
-    <mergeCell ref="D59:D69"/>
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="G5:G6"/>
-    <mergeCell ref="H5:H6"/>
-    <mergeCell ref="B2:B93"/>
-    <mergeCell ref="C2:C9"/>
-    <mergeCell ref="C35:C93"/>
-    <mergeCell ref="D70:D89"/>
-    <mergeCell ref="D90:D93"/>
   </mergeCells>
+  <conditionalFormatting sqref="H2 H4:H5 H7:H12 H14:H93">
+    <cfRule type="expression" dxfId="7" priority="1">
+      <formula>$H2&lt;=2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="6" priority="2">
+      <formula>$H2&lt;=4</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="5" priority="3">
+      <formula>$H2&gt;4</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J2:L93">
+    <cfRule type="expression" dxfId="4" priority="4">
+      <formula>$I2="Non"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="K2:K93">
-    <cfRule type="expression" dxfId="7" priority="6">
+    <cfRule type="expression" dxfId="3" priority="6">
       <formula>$K2="KO"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="7">
+    <cfRule type="expression" dxfId="2" priority="7">
       <formula>$K2="OK"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="8">
+    <cfRule type="expression" dxfId="1" priority="8">
       <formula>$K2="NT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L2:L93">
-    <cfRule type="expression" dxfId="4" priority="5">
+    <cfRule type="expression" dxfId="0" priority="5">
       <formula>$K2&lt;&gt;"OK"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J2:L93">
-    <cfRule type="expression" dxfId="3" priority="4">
-      <formula>$I2="Non"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H2 H4:H5 H7:H12 H14:H93">
-    <cfRule type="expression" dxfId="2" priority="1">
-      <formula>$H2&lt;=2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="1" priority="2">
-      <formula>$H2&lt;=4</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="0" priority="3">
-      <formula>$H2&gt;4</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
@@ -4102,10 +4099,10 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="30"/>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
+      <c r="A2" s="44"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
     </row>
     <row r="3" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="21"/>
@@ -4116,34 +4113,34 @@
       <c r="A4" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="28" t="s">
+      <c r="B4" s="46" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="29"/>
+      <c r="C4" s="47"/>
       <c r="D4" s="23" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B5" s="26"/>
-      <c r="C5" s="27"/>
+      <c r="B5" s="45"/>
+      <c r="C5" s="43"/>
       <c r="D5" s="24"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="65" t="s">
+      <c r="B6" s="48" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="66"/>
+      <c r="C6" s="49"/>
       <c r="D6" s="9" t="s">
         <v>222</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B7" s="26"/>
-      <c r="C7" s="27"/>
+      <c r="B7" s="45"/>
+      <c r="C7" s="43"/>
       <c r="D7" s="24"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -4160,14 +4157,14 @@
         <v>223</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A9" s="17" t="s">
         <v>15</v>
       </c>
       <c r="B9" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="67" t="s">
+      <c r="C9" s="17" t="s">
         <v>12</v>
       </c>
       <c r="D9" s="18" t="s">
@@ -4189,7 +4186,7 @@
       </c>
     </row>
     <row r="11" spans="1:4" s="15" customFormat="1" ht="201.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="27" t="s">
+      <c r="A11" s="43" t="s">
         <v>17</v>
       </c>
       <c r="B11" s="14" t="s">
@@ -4203,7 +4200,7 @@
       </c>
     </row>
     <row r="12" spans="1:4" ht="201.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="27"/>
+      <c r="A12" s="43"/>
       <c r="B12" s="14" t="s">
         <v>219</v>
       </c>
@@ -4213,7 +4210,7 @@
       </c>
     </row>
     <row r="13" spans="1:4" ht="244.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="27"/>
+      <c r="A13" s="43"/>
       <c r="B13" s="14" t="s">
         <v>220</v>
       </c>
@@ -4248,7 +4245,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="28" t="s">
         <v>124</v>
       </c>
       <c r="B1"/>
@@ -4263,55 +4260,55 @@
       <c r="D2" s="2"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="51" t="s">
+      <c r="A3" s="34" t="s">
         <v>126</v>
       </c>
-      <c r="B3" s="51" t="s">
+      <c r="B3" s="34" t="s">
         <v>127</v>
       </c>
-      <c r="C3" s="51" t="s">
+      <c r="C3" s="34" t="s">
         <v>3</v>
       </c>
       <c r="D3" s="2"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="52" t="s">
+      <c r="A4" s="35" t="s">
         <v>128</v>
       </c>
-      <c r="B4" s="53"/>
-      <c r="C4" s="54"/>
+      <c r="B4" s="65"/>
+      <c r="C4" s="66"/>
       <c r="D4" s="2"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="52" t="s">
+      <c r="A5" s="35" t="s">
         <v>129</v>
       </c>
-      <c r="B5" s="53"/>
-      <c r="C5" s="54"/>
+      <c r="B5" s="65"/>
+      <c r="C5" s="66"/>
       <c r="D5" s="2"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="52">
+      <c r="A6" s="35">
         <v>1</v>
       </c>
-      <c r="B6" s="52"/>
-      <c r="C6" s="52"/>
+      <c r="B6" s="35"/>
+      <c r="C6" s="35"/>
       <c r="D6" s="2"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="52">
+      <c r="A7" s="35">
         <v>2</v>
       </c>
-      <c r="B7" s="52"/>
-      <c r="C7" s="52"/>
+      <c r="B7" s="35"/>
+      <c r="C7" s="35"/>
       <c r="D7" s="2"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="52">
+      <c r="A8" s="35">
         <v>3</v>
       </c>
-      <c r="B8" s="52"/>
-      <c r="C8" s="52"/>
+      <c r="B8" s="35"/>
+      <c r="C8" s="35"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9"/>
@@ -4324,7 +4321,7 @@
       <c r="C10"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="45" t="s">
+      <c r="A11" s="28" t="s">
         <v>130</v>
       </c>
       <c r="B11"/>
@@ -4338,50 +4335,50 @@
       <c r="C12"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="51" t="s">
+      <c r="A13" s="34" t="s">
         <v>126</v>
       </c>
-      <c r="B13" s="51" t="s">
+      <c r="B13" s="34" t="s">
         <v>127</v>
       </c>
-      <c r="C13" s="51" t="s">
+      <c r="C13" s="34" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" s="52" t="s">
+      <c r="A14" s="35" t="s">
         <v>128</v>
       </c>
-      <c r="B14" s="52"/>
-      <c r="C14" s="52"/>
+      <c r="B14" s="35"/>
+      <c r="C14" s="35"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" s="52" t="s">
+      <c r="A15" s="35" t="s">
         <v>129</v>
       </c>
-      <c r="B15" s="52"/>
-      <c r="C15" s="52"/>
+      <c r="B15" s="35"/>
+      <c r="C15" s="35"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="52">
+      <c r="A16" s="35">
         <v>1</v>
       </c>
-      <c r="B16" s="52"/>
-      <c r="C16" s="52"/>
+      <c r="B16" s="35"/>
+      <c r="C16" s="35"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="52">
+      <c r="A17" s="35">
         <v>2</v>
       </c>
-      <c r="B17" s="52"/>
-      <c r="C17" s="52"/>
+      <c r="B17" s="35"/>
+      <c r="C17" s="35"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="52">
+      <c r="A18" s="35">
         <v>3</v>
       </c>
-      <c r="B18" s="52"/>
-      <c r="C18" s="52"/>
+      <c r="B18" s="35"/>
+      <c r="C18" s="35"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19"/>
@@ -4394,7 +4391,7 @@
       <c r="C20"/>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="45" t="s">
+      <c r="A21" s="28" t="s">
         <v>131</v>
       </c>
       <c r="B21"/>
@@ -4408,50 +4405,50 @@
       <c r="C22"/>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="51" t="s">
+      <c r="A23" s="34" t="s">
         <v>126</v>
       </c>
-      <c r="B23" s="51" t="s">
+      <c r="B23" s="34" t="s">
         <v>127</v>
       </c>
-      <c r="C23" s="51" t="s">
+      <c r="C23" s="34" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="52" t="s">
+      <c r="A24" s="35" t="s">
         <v>128</v>
       </c>
-      <c r="B24" s="52"/>
-      <c r="C24" s="52"/>
+      <c r="B24" s="35"/>
+      <c r="C24" s="35"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="52" t="s">
+      <c r="A25" s="35" t="s">
         <v>129</v>
       </c>
-      <c r="B25" s="52"/>
-      <c r="C25" s="52"/>
+      <c r="B25" s="35"/>
+      <c r="C25" s="35"/>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="52">
+      <c r="A26" s="35">
         <v>1</v>
       </c>
-      <c r="B26" s="52"/>
-      <c r="C26" s="52"/>
+      <c r="B26" s="35"/>
+      <c r="C26" s="35"/>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" s="52">
+      <c r="A27" s="35">
         <v>2</v>
       </c>
-      <c r="B27" s="52"/>
-      <c r="C27" s="52"/>
+      <c r="B27" s="35"/>
+      <c r="C27" s="35"/>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" s="52">
+      <c r="A28" s="35">
         <v>3</v>
       </c>
-      <c r="B28" s="52"/>
-      <c r="C28" s="52"/>
+      <c r="B28" s="35"/>
+      <c r="C28" s="35"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4475,15 +4472,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100DE74238BD041D74DA6DBFAB08BDAD7AF" ma:contentTypeVersion="11" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="bcd70524c02bcffc8b441d1fc1dca0cc">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="62a23633-e9fe-47f7-a756-540d8a70e647" xmlns:ns3="fa25dd69-b1ca-48f4-a209-94e3282b6cc7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fb0f7e4e371af128dcbef8683eb2728a" ns2:_="" ns3:_="">
     <xsd:import namespace="62a23633-e9fe-47f7-a756-540d8a70e647"/>
@@ -4678,6 +4666,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{715B483B-C49B-42BD-85E3-8B799FA115A1}">
   <ds:schemaRefs>
@@ -4692,14 +4689,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9663E150-767C-45B7-A45E-CD530BED6AC8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{798DAF4D-4D9E-44FE-B80E-1EFB817FD3CF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4716,4 +4705,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9663E150-767C-45B7-A45E-CD530BED6AC8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>